<commit_message>
fix: extend staff SUM range to H200 so manually added rows are included
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Colombia_Teams.xlsx
+++ b/Colombia_Teams.xlsx
@@ -1890,7 +1890,7 @@
         <v/>
       </c>
       <c r="G3" s="32">
-        <f>SUM(Staff!H4:Staff!H7)</f>
+        <f>SUM(Staff!H4:Staff!H200)</f>
         <v/>
       </c>
       <c r="H3" s="32">
@@ -1975,7 +1975,7 @@
         <v/>
       </c>
       <c r="G4" s="32">
-        <f>SUM(Staff!I4:Staff!I7)</f>
+        <f>SUM(Staff!I4:Staff!I200)</f>
         <v/>
       </c>
       <c r="H4" s="32">
@@ -2060,7 +2060,7 @@
         <v/>
       </c>
       <c r="G5" s="32">
-        <f>SUM(Staff!H4:Staff!H7)</f>
+        <f>SUM(Staff!H4:Staff!H200)</f>
         <v/>
       </c>
       <c r="H5" s="32">
@@ -2145,7 +2145,7 @@
         <v/>
       </c>
       <c r="G6" s="32">
-        <f>SUM(Staff!I4:Staff!I7)</f>
+        <f>SUM(Staff!I4:Staff!I200)</f>
         <v/>
       </c>
       <c r="H6" s="32">

</xml_diff>